<commit_message>
Add product-filter, support-products, video-embed blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/product-filter/product-filter.css
- blocks/product-filter/product-filter.js
- blocks/support-products/support-products.css
- blocks/video-embed/video-embed.css
- blocks/video-embed/video-embed.js
- styles/styles.css
- tools/importer/reports/ark.report.json
- tools/importer/reports/import-category-directory.report.xlsx
- tools/importer/reports/partner-alliance/overview.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-category-directory.report.xlsx
+++ b/tools/importer/reports/import-category-directory.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="206">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>category-directory</t>
   </si>
   <si>
-    <t>2026-04-05T11:50:08.226Z</t>
+    <t>2026-04-05T16:31:53.358Z</t>
   </si>
   <si>
     <t>Intel® Product Specifications</t>
@@ -211,7 +211,7 @@
     <t>company-overview/company-overview</t>
   </si>
   <si>
-    <t>2026-04-03T21:01:07.254Z</t>
+    <t>2026-04-05T11:50:47.858Z</t>
   </si>
   <si>
     <t>Innovation starts here</t>
@@ -268,6 +268,21 @@
     <t>https://www.intel.com/content/www/us/en/developer/overview.html</t>
   </si>
   <si>
+    <t>download-center/home.report.json</t>
+  </si>
+  <si>
+    <t>download-center/home</t>
+  </si>
+  <si>
+    <t>2026-04-05T11:50:37.419Z</t>
+  </si>
+  <si>
+    <t>Download Intel Drivers and Software</t>
+  </si>
+  <si>
+    <t>https://www.intel.com/content/www/us/en/download-center/home.html</t>
+  </si>
+  <si>
     <t>edge-computing/overview.report.json</t>
   </si>
   <si>
@@ -295,7 +310,7 @@
     <t>environment/sustainability</t>
   </si>
   <si>
-    <t>2026-04-03T20:58:58.658Z</t>
+    <t>2026-04-05T11:50:28.479Z</t>
   </si>
   <si>
     <t>Sustainable Computing for a Sustainable Future</t>
@@ -304,6 +319,24 @@
     <t>https://www.intel.com/content/www/us/en/environment/sustainability.html</t>
   </si>
   <si>
+    <t>foundry/overview.report.json</t>
+  </si>
+  <si>
+    <t>["cards-product","cards-product","columns","columns"]</t>
+  </si>
+  <si>
+    <t>foundry/overview</t>
+  </si>
+  <si>
+    <t>2026-04-05T11:50:33.656Z</t>
+  </si>
+  <si>
+    <t>Semiconductor Manufacturing Company for the AI Era</t>
+  </si>
+  <si>
+    <t>https://www.intel.com/content/www/us/en/foundry/overview.html</t>
+  </si>
+  <si>
     <t>gaming/esports.report.json</t>
   </si>
   <si>
@@ -391,6 +424,24 @@
     <t>https://www.intel.com/content/www/us/en/high-performance-computing/overview.html</t>
   </si>
   <si>
+    <t>jobs/life-at-intel.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards-news"]</t>
+  </si>
+  <si>
+    <t>jobs/life-at-intel</t>
+  </si>
+  <si>
+    <t>2026-04-05T11:50:53.581Z</t>
+  </si>
+  <si>
+    <t>Work and Life at Intel</t>
+  </si>
+  <si>
+    <t>https://www.intel.com/content/www/us/en/jobs/life-at-intel.html</t>
+  </si>
+  <si>
     <t>manufacturing/manufacturing-industrial-overview.report.json</t>
   </si>
   <si>
@@ -415,7 +466,7 @@
     <t>partner-alliance/overview</t>
   </si>
   <si>
-    <t>2026-04-05T11:50:18.817Z</t>
+    <t>2026-04-05T16:55:38.134Z</t>
   </si>
   <si>
     <t>Intel® Partner Alliance</t>
@@ -442,16 +493,34 @@
     <t>security/overview.report.json</t>
   </si>
   <si>
+    <t>["hero","cards-product","cards-product","cards-product","cards-product","cards-product","cards-product","cards-product","columns"]</t>
+  </si>
+  <si>
     <t>security/overview</t>
   </si>
   <si>
-    <t>2026-04-03T21:00:17.973Z</t>
+    <t>2026-04-05T11:50:23.414Z</t>
   </si>
   <si>
     <t>Security Innovation for Business Networks | Intel®</t>
   </si>
   <si>
     <t>https://www.intel.com/content/www/us/en/security/overview.html</t>
+  </si>
+  <si>
+    <t>support/detect.report.json</t>
+  </si>
+  <si>
+    <t>support/detect</t>
+  </si>
+  <si>
+    <t>2026-04-05T11:50:41.779Z</t>
+  </si>
+  <si>
+    <t>Intel® Driver &amp; Support Assistant</t>
+  </si>
+  <si>
+    <t>https://www.intel.com/content/www/us/en/support/detect.html</t>
   </si>
   <si>
     <t>topics/overview.report.json</t>
@@ -948,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1326,36 +1395,36 @@
         <v>85</v>
       </c>
       <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>86</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
         <v>87</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>88</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>89</v>
-      </c>
-      <c r="H15" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" t="s">
         <v>91</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>92</v>
-      </c>
-      <c r="C16" t="s">
-        <v>93</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1364,24 +1433,24 @@
         <v>32</v>
       </c>
       <c r="F16" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" t="s">
         <v>94</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>95</v>
-      </c>
-      <c r="H16" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
         <v>97</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>98</v>
-      </c>
-      <c r="C17" t="s">
-        <v>99</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1390,24 +1459,24 @@
         <v>32</v>
       </c>
       <c r="F17" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" t="s">
         <v>100</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>101</v>
-      </c>
-      <c r="H17" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
         <v>103</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>104</v>
-      </c>
-      <c r="C18" t="s">
-        <v>105</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1416,24 +1485,24 @@
         <v>32</v>
       </c>
       <c r="F18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>107</v>
-      </c>
-      <c r="H18" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
         <v>109</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>110</v>
-      </c>
-      <c r="C19" t="s">
-        <v>111</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -1442,24 +1511,24 @@
         <v>32</v>
       </c>
       <c r="F19" t="s">
+        <v>111</v>
+      </c>
+      <c r="G19" t="s">
         <v>112</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>113</v>
-      </c>
-      <c r="H19" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>114</v>
+      </c>
+      <c r="B20" t="s">
         <v>115</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>116</v>
-      </c>
-      <c r="C20" t="s">
-        <v>117</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
@@ -1468,21 +1537,21 @@
         <v>32</v>
       </c>
       <c r="F20" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" t="s">
         <v>118</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>119</v>
-      </c>
-      <c r="H20" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" t="s">
         <v>121</v>
-      </c>
-      <c r="B21" t="s">
-        <v>9</v>
       </c>
       <c r="C21" t="s">
         <v>122</v>
@@ -1491,7 +1560,7 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F21" t="s">
         <v>123</v>
@@ -1560,62 +1629,62 @@
         <v>137</v>
       </c>
       <c r="B24" t="s">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="C24" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F24" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B25" t="s">
-        <v>9</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F25" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G25" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H25" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
@@ -1624,24 +1693,24 @@
         <v>12</v>
       </c>
       <c r="F26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H26" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
@@ -1650,76 +1719,76 @@
         <v>12</v>
       </c>
       <c r="F27" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H27" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B28" t="s">
-        <v>9</v>
+        <v>160</v>
       </c>
       <c r="C28" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F28" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G28" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H28" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G29" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H29" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
@@ -1728,65 +1797,169 @@
         <v>12</v>
       </c>
       <c r="F30" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G30" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H30" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="F31" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G31" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H31" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B32" t="s">
-        <v>178</v>
+        <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" t="s">
+        <v>182</v>
+      </c>
+      <c r="G32" t="s">
+        <v>183</v>
+      </c>
+      <c r="H32" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>185</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>186</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" t="s">
+        <v>187</v>
+      </c>
+      <c r="G33" t="s">
+        <v>188</v>
+      </c>
+      <c r="H33" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>191</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" t="s">
+        <v>192</v>
+      </c>
+      <c r="G34" t="s">
+        <v>193</v>
+      </c>
+      <c r="H34" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>196</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
         <v>32</v>
       </c>
-      <c r="F32" t="s">
-        <v>180</v>
-      </c>
-      <c r="G32" t="s">
-        <v>181</v>
-      </c>
-      <c r="H32" t="s">
-        <v>182</v>
+      <c r="F35" t="s">
+        <v>197</v>
+      </c>
+      <c r="G35" t="s">
+        <v>198</v>
+      </c>
+      <c r="H35" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>200</v>
+      </c>
+      <c r="B36" t="s">
+        <v>201</v>
+      </c>
+      <c r="C36" t="s">
+        <v>202</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" t="s">
+        <v>203</v>
+      </c>
+      <c r="G36" t="s">
+        <v>204</v>
+      </c>
+      <c r="H36" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>